<commit_message>
docs: fix proje kontrol listesi
</commit_message>
<xml_diff>
--- a/docs/Proje_Kontrol_Listesi_482.xlsx
+++ b/docs/Proje_Kontrol_Listesi_482.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akife\OneDrive\Masaüstü\wish-list\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E2F5C9-D42D-4CFD-AA74-C706E3F6B35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Detayl__Kontrol_Listesi" sheetId="1" r:id="rId4"/>
+    <sheet name="Detayl__Kontrol_Listesi" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="KW2K0TsaGXyvPzKK2+RsV0KpwQiD1cCYWqdBNZIAGvo="/>
@@ -396,9 +405,6 @@
     <t>Ek gereksinimler açıkça listelenmiş mi?</t>
   </si>
   <si>
-    <t>Software_Requirements_Document.pdf, Sayfa 9, Bölüm 4.5 (Legal and Ethical Constraints)</t>
-  </si>
-  <si>
     <t>Yasal ve etik gereksinimler: KVKK (Kişisel Verilerin Korunması Kanunu) ve GDPR kapsamında veri gizliliği sağlanmaktadır. Etik kazıma standartları çerçevesinde aynı domaine ardışık istekler arasında minimum 2 saniye gecikme uygulanmaktadır. Sistem yalnızca kamuya açık meta verilere erişmekte; üçüncü taraf platformların fikri mülkiyetine saygı gösterilmektedir. Proje son teslim tarihi akademik dönem takvimi ile sınırlıdır.</t>
   </si>
   <si>
@@ -435,9 +441,6 @@
     <t>Yazılım kalite güvence planı tanımlanmış mı? amac, kapsam, kalite hedefleri, uygulanacak standartlar, sqa aktiviteleri (kod inceleme, test, surec denetimi, hata izleme etc.), sorumluluklar, dogrulama ve gecerleme, hata ve degisiklik yonetimi, test planlari ve kriterleri, raporlama ve kayit tutma</t>
   </si>
   <si>
-    <t>Delta_Design_Report.pdf, Sayfa 3, Bölüm 4 (Impact on Quality Metrics and Testing), Delta_Design_Report.pdf, Sayfa 4, Bölüm 6 (Software Quality Assurance Plan (SQAP))</t>
-  </si>
-  <si>
     <t>Kalite güvencesi kapsamında Observer ve Factory örüntülerine yönelik mimari kararlılık testleri yazılmıştır (test_scraper_factory.py, test_patterns.py, test_category_factory.py). Kalite boyutları değerlendirilmiştir: Modülerlik/Bağlaşım (PriceMonitor ile TargetPriceNotificationObserver ayrıştırması), Verimlilik (frekans farkındalıklı zamanlama), Güvenilirlik (codec hatası düzeltmesi) ve Tasarım Uygunluğu (CategoryFactory ve ScraperFactory örüntü düzeltmeleri). FastAPI TestClient API endpoint testleri için kullanılabilmektedir.</t>
   </si>
   <si>
@@ -568,44 +571,50 @@
   </si>
   <si>
     <t>Yasal ve etik uyumluluk üç temel alanda ele alınmıştır: (1) Veri Gizliliği (KVKK/GDPR) – Supabase Auth aracılığıyla yalnızca e-posta adresi toplanmakta, finansal veya hassas kişisel veri saklanmamaktadır; (2) Etik Kazıma Standartları – üçüncü taraf platformların fikri mülkiyetine ve altyapısına saygı göstermek amacıyla ardışık istekler arasında minimum 2 saniye gecikme uygulanmaktadır; (3) Şeffaflık – sistem yalnızca kamuya açık meta verilere erişmekte, ödeme duvarları veya kimlik doğrulama katmanları aşılmaya çalışılmamaktadır.</t>
+  </si>
+  <si>
+    <t>Software_Requirements_Document.pdf, Sayfa 20, Bölüm 11 (Other Requirements)</t>
+  </si>
+  <si>
+    <t>Delta_Design_Report.pdf, Sayfa 3, Bölüm 4 (Impact on Quality Metrics and Testing), Delta_Design_Report.docx.pdf, Sayfa 4, Bölüm 6 ( Software Quality Assurance Plan (SQAP))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <u/>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Times New Roman"/>
     </font>
@@ -615,62 +624,68 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -860,27 +875,30 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <dimension ref="A1:F1000"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="43.0"/>
-    <col customWidth="1" min="2" max="2" width="57.75"/>
-    <col customWidth="1" min="3" max="3" width="46.38"/>
-    <col customWidth="1" min="4" max="4" width="45.25"/>
-    <col customWidth="1" min="5" max="5" width="23.25"/>
-    <col customWidth="1" min="6" max="6" width="24.75"/>
-    <col customWidth="1" min="7" max="26" width="12.75"/>
+    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="2" max="2" width="57.77734375" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="45.21875" customWidth="1"/>
+    <col min="5" max="5" width="23.21875" customWidth="1"/>
+    <col min="6" max="6" width="24.77734375" customWidth="1"/>
+    <col min="7" max="26" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +909,7 @@
       <c r="D1" s="2"/>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -902,7 +920,7 @@
       <c r="D2" s="2"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -920,7 +938,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" ht="79.5" customHeight="1">
+    <row r="4" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
@@ -938,7 +956,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" ht="79.5" customHeight="1">
+    <row r="5" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>14</v>
       </c>
@@ -956,7 +974,7 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" ht="79.5" customHeight="1">
+    <row r="6" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -974,7 +992,7 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" ht="79.5" customHeight="1">
+    <row r="7" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
@@ -992,7 +1010,7 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" ht="79.5" customHeight="1">
+    <row r="8" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>26</v>
       </c>
@@ -1010,7 +1028,7 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" ht="79.5" customHeight="1">
+    <row r="9" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>30</v>
       </c>
@@ -1028,7 +1046,7 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" ht="79.5" customHeight="1">
+    <row r="10" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>34</v>
       </c>
@@ -1046,7 +1064,7 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" ht="79.5" customHeight="1">
+    <row r="11" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>38</v>
       </c>
@@ -1064,7 +1082,7 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" ht="79.5" customHeight="1">
+    <row r="12" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>43</v>
       </c>
@@ -1082,7 +1100,7 @@
       </c>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" ht="79.5" customHeight="1">
+    <row r="13" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>48</v>
       </c>
@@ -1100,7 +1118,7 @@
       </c>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" ht="79.5" customHeight="1">
+    <row r="14" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>52</v>
       </c>
@@ -1118,7 +1136,7 @@
       </c>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" ht="79.5" customHeight="1">
+    <row r="15" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>57</v>
       </c>
@@ -1136,7 +1154,7 @@
       </c>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" ht="79.5" customHeight="1">
+    <row r="16" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>61</v>
       </c>
@@ -1154,7 +1172,7 @@
       </c>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" ht="79.5" customHeight="1">
+    <row r="17" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>65</v>
       </c>
@@ -1172,7 +1190,7 @@
       </c>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" ht="79.5" customHeight="1">
+    <row r="18" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>69</v>
       </c>
@@ -1190,7 +1208,7 @@
       </c>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" ht="79.5" customHeight="1">
+    <row r="19" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>74</v>
       </c>
@@ -1208,7 +1226,7 @@
       </c>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" ht="79.5" customHeight="1">
+    <row r="20" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>78</v>
       </c>
@@ -1226,7 +1244,7 @@
       </c>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" ht="79.5" customHeight="1">
+    <row r="21" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>82</v>
       </c>
@@ -1244,7 +1262,7 @@
       </c>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" ht="79.5" customHeight="1">
+    <row r="22" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>87</v>
       </c>
@@ -1262,7 +1280,7 @@
       </c>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" ht="79.5" customHeight="1">
+    <row r="23" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>91</v>
       </c>
@@ -1280,7 +1298,7 @@
       </c>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" ht="79.5" customHeight="1">
+    <row r="24" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>96</v>
       </c>
@@ -1298,7 +1316,7 @@
       </c>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" ht="79.5" customHeight="1">
+    <row r="25" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>101</v>
       </c>
@@ -1316,7 +1334,7 @@
       </c>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" ht="79.5" customHeight="1">
+    <row r="26" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>106</v>
       </c>
@@ -1324,2218 +1342,2217 @@
         <v>107</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>108</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>109</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" ht="79.5" customHeight="1">
+    <row r="27" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="D27" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F27" s="3"/>
-    </row>
-    <row r="28" ht="79.5" customHeight="1">
-      <c r="A28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="D28" s="7" t="s">
         <v>117</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>118</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" ht="79.5" customHeight="1">
+    <row r="29" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="E29" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="F29" s="3"/>
+    </row>
+    <row r="30" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="B30" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F29" s="3"/>
-    </row>
-    <row r="30" ht="79.5" customHeight="1">
-      <c r="A30" s="5" t="s">
+      <c r="C30" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="D30" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="E30" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="F30" s="3"/>
+    </row>
+    <row r="31" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="B31" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F30" s="3"/>
-    </row>
-    <row r="31" ht="79.5" customHeight="1">
-      <c r="A31" s="5" t="s">
+      <c r="C31" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="E31" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="F31" s="3"/>
+    </row>
+    <row r="32" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="B32" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" ht="79.5" customHeight="1">
-      <c r="A32" s="5" t="s">
+      <c r="C32" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>135</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>137</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" ht="79.5" customHeight="1">
+    <row r="33" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="D33" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>141</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" ht="79.5" customHeight="1">
+    <row r="34" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="D34" s="7" t="s">
         <v>143</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>145</v>
       </c>
       <c r="E34" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" ht="79.5" customHeight="1">
+    <row r="35" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="D35" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>149</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" ht="79.5" customHeight="1">
+    <row r="36" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="D36" s="7" t="s">
         <v>151</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>153</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" ht="79.5" customHeight="1">
+    <row r="37" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="D37" s="7" t="s">
         <v>155</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>157</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" ht="79.5" customHeight="1">
+    <row r="38" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="D38" s="7" t="s">
         <v>159</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>161</v>
       </c>
       <c r="E38" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" ht="79.5" customHeight="1">
+    <row r="39" spans="1:6" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="D39" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>165</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
+    <row r="76" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
+    <row r="77" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" ht="15.75" customHeight="1">
+    <row r="78" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
+    <row r="79" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" ht="15.75" customHeight="1">
+    <row r="80" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1">
+    <row r="81" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
+    <row r="82" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1">
+    <row r="83" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" ht="15.75" customHeight="1">
+    <row r="84" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
+    <row r="85" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
+    <row r="86" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
+    <row r="87" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
+    <row r="88" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
+    <row r="89" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" ht="15.75" customHeight="1">
+    <row r="90" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
+    <row r="91" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" ht="15.75" customHeight="1">
+    <row r="92" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
+    <row r="93" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
+    <row r="94" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
+    <row r="95" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
+    <row r="96" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
+    <row r="97" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" ht="15.75" customHeight="1">
+    <row r="98" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
+    <row r="99" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
+    <row r="100" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" ht="15.75" customHeight="1">
+    <row r="101" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
       <c r="F101" s="3"/>
     </row>
-    <row r="102" ht="15.75" customHeight="1">
+    <row r="102" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
       <c r="F102" s="3"/>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
+    <row r="103" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="F103" s="3"/>
     </row>
-    <row r="104" ht="15.75" customHeight="1">
+    <row r="104" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="F104" s="3"/>
     </row>
-    <row r="105" ht="15.75" customHeight="1">
+    <row r="105" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
       <c r="F105" s="3"/>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
+    <row r="106" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="F106" s="3"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
+    <row r="107" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="F107" s="3"/>
     </row>
-    <row r="108" ht="15.75" customHeight="1">
+    <row r="108" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="F108" s="3"/>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
+    <row r="109" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
       <c r="F109" s="3"/>
     </row>
-    <row r="110" ht="15.75" customHeight="1">
+    <row r="110" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="F110" s="3"/>
     </row>
-    <row r="111" ht="15.75" customHeight="1">
+    <row r="111" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="F111" s="3"/>
     </row>
-    <row r="112" ht="15.75" customHeight="1">
+    <row r="112" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="F112" s="3"/>
     </row>
-    <row r="113" ht="15.75" customHeight="1">
+    <row r="113" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="F113" s="3"/>
     </row>
-    <row r="114" ht="15.75" customHeight="1">
+    <row r="114" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
       <c r="F114" s="3"/>
     </row>
-    <row r="115" ht="15.75" customHeight="1">
+    <row r="115" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
       <c r="F115" s="3"/>
     </row>
-    <row r="116" ht="15.75" customHeight="1">
+    <row r="116" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
       <c r="F116" s="3"/>
     </row>
-    <row r="117" ht="15.75" customHeight="1">
+    <row r="117" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
       <c r="F117" s="3"/>
     </row>
-    <row r="118" ht="15.75" customHeight="1">
+    <row r="118" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="F118" s="3"/>
     </row>
-    <row r="119" ht="15.75" customHeight="1">
+    <row r="119" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="F119" s="3"/>
     </row>
-    <row r="120" ht="15.75" customHeight="1">
+    <row r="120" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="F120" s="3"/>
     </row>
-    <row r="121" ht="15.75" customHeight="1">
+    <row r="121" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
       <c r="F121" s="3"/>
     </row>
-    <row r="122" ht="15.75" customHeight="1">
+    <row r="122" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
       <c r="F122" s="3"/>
     </row>
-    <row r="123" ht="15.75" customHeight="1">
+    <row r="123" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="F123" s="3"/>
     </row>
-    <row r="124" ht="15.75" customHeight="1">
+    <row r="124" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="F124" s="3"/>
     </row>
-    <row r="125" ht="15.75" customHeight="1">
+    <row r="125" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="F125" s="3"/>
     </row>
-    <row r="126" ht="15.75" customHeight="1">
+    <row r="126" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="F126" s="3"/>
     </row>
-    <row r="127" ht="15.75" customHeight="1">
+    <row r="127" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
       <c r="F127" s="3"/>
     </row>
-    <row r="128" ht="15.75" customHeight="1">
+    <row r="128" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
       <c r="F128" s="3"/>
     </row>
-    <row r="129" ht="15.75" customHeight="1">
+    <row r="129" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="F129" s="3"/>
     </row>
-    <row r="130" ht="15.75" customHeight="1">
+    <row r="130" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
       <c r="F130" s="3"/>
     </row>
-    <row r="131" ht="15.75" customHeight="1">
+    <row r="131" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="F131" s="3"/>
     </row>
-    <row r="132" ht="15.75" customHeight="1">
+    <row r="132" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="F132" s="3"/>
     </row>
-    <row r="133" ht="15.75" customHeight="1">
+    <row r="133" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="F133" s="3"/>
     </row>
-    <row r="134" ht="15.75" customHeight="1">
+    <row r="134" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="F134" s="3"/>
     </row>
-    <row r="135" ht="15.75" customHeight="1">
+    <row r="135" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="F135" s="3"/>
     </row>
-    <row r="136" ht="15.75" customHeight="1">
+    <row r="136" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="F136" s="3"/>
     </row>
-    <row r="137" ht="15.75" customHeight="1">
+    <row r="137" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
       <c r="F137" s="3"/>
     </row>
-    <row r="138" ht="15.75" customHeight="1">
+    <row r="138" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
       <c r="F138" s="3"/>
     </row>
-    <row r="139" ht="15.75" customHeight="1">
+    <row r="139" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
       <c r="F139" s="3"/>
     </row>
-    <row r="140" ht="15.75" customHeight="1">
+    <row r="140" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
       <c r="F140" s="3"/>
     </row>
-    <row r="141" ht="15.75" customHeight="1">
+    <row r="141" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
       <c r="F141" s="3"/>
     </row>
-    <row r="142" ht="15.75" customHeight="1">
+    <row r="142" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
       <c r="F142" s="3"/>
     </row>
-    <row r="143" ht="15.75" customHeight="1">
+    <row r="143" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
       <c r="F143" s="3"/>
     </row>
-    <row r="144" ht="15.75" customHeight="1">
+    <row r="144" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
       <c r="F144" s="3"/>
     </row>
-    <row r="145" ht="15.75" customHeight="1">
+    <row r="145" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
       <c r="F145" s="3"/>
     </row>
-    <row r="146" ht="15.75" customHeight="1">
+    <row r="146" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
       <c r="F146" s="3"/>
     </row>
-    <row r="147" ht="15.75" customHeight="1">
+    <row r="147" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
       <c r="F147" s="3"/>
     </row>
-    <row r="148" ht="15.75" customHeight="1">
+    <row r="148" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
       <c r="F148" s="3"/>
     </row>
-    <row r="149" ht="15.75" customHeight="1">
+    <row r="149" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
       <c r="F149" s="3"/>
     </row>
-    <row r="150" ht="15.75" customHeight="1">
+    <row r="150" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
       <c r="F150" s="3"/>
     </row>
-    <row r="151" ht="15.75" customHeight="1">
+    <row r="151" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
       <c r="F151" s="3"/>
     </row>
-    <row r="152" ht="15.75" customHeight="1">
+    <row r="152" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
       <c r="F152" s="3"/>
     </row>
-    <row r="153" ht="15.75" customHeight="1">
+    <row r="153" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
       <c r="F153" s="3"/>
     </row>
-    <row r="154" ht="15.75" customHeight="1">
+    <row r="154" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
       <c r="F154" s="3"/>
     </row>
-    <row r="155" ht="15.75" customHeight="1">
+    <row r="155" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
       <c r="F155" s="3"/>
     </row>
-    <row r="156" ht="15.75" customHeight="1">
+    <row r="156" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
       <c r="F156" s="3"/>
     </row>
-    <row r="157" ht="15.75" customHeight="1">
+    <row r="157" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
       <c r="D157" s="3"/>
       <c r="F157" s="3"/>
     </row>
-    <row r="158" ht="15.75" customHeight="1">
+    <row r="158" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
       <c r="D158" s="3"/>
       <c r="F158" s="3"/>
     </row>
-    <row r="159" ht="15.75" customHeight="1">
+    <row r="159" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
       <c r="F159" s="3"/>
     </row>
-    <row r="160" ht="15.75" customHeight="1">
+    <row r="160" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
       <c r="F160" s="3"/>
     </row>
-    <row r="161" ht="15.75" customHeight="1">
+    <row r="161" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
       <c r="D161" s="3"/>
       <c r="F161" s="3"/>
     </row>
-    <row r="162" ht="15.75" customHeight="1">
+    <row r="162" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
       <c r="D162" s="3"/>
       <c r="F162" s="3"/>
     </row>
-    <row r="163" ht="15.75" customHeight="1">
+    <row r="163" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
       <c r="F163" s="3"/>
     </row>
-    <row r="164" ht="15.75" customHeight="1">
+    <row r="164" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
       <c r="F164" s="3"/>
     </row>
-    <row r="165" ht="15.75" customHeight="1">
+    <row r="165" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
       <c r="D165" s="3"/>
       <c r="F165" s="3"/>
     </row>
-    <row r="166" ht="15.75" customHeight="1">
+    <row r="166" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
       <c r="D166" s="3"/>
       <c r="F166" s="3"/>
     </row>
-    <row r="167" ht="15.75" customHeight="1">
+    <row r="167" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
       <c r="F167" s="3"/>
     </row>
-    <row r="168" ht="15.75" customHeight="1">
+    <row r="168" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
       <c r="D168" s="3"/>
       <c r="F168" s="3"/>
     </row>
-    <row r="169" ht="15.75" customHeight="1">
+    <row r="169" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
       <c r="D169" s="3"/>
       <c r="F169" s="3"/>
     </row>
-    <row r="170" ht="15.75" customHeight="1">
+    <row r="170" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
       <c r="D170" s="3"/>
       <c r="F170" s="3"/>
     </row>
-    <row r="171" ht="15.75" customHeight="1">
+    <row r="171" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
       <c r="D171" s="3"/>
       <c r="F171" s="3"/>
     </row>
-    <row r="172" ht="15.75" customHeight="1">
+    <row r="172" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
       <c r="F172" s="3"/>
     </row>
-    <row r="173" ht="15.75" customHeight="1">
+    <row r="173" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
       <c r="D173" s="3"/>
       <c r="F173" s="3"/>
     </row>
-    <row r="174" ht="15.75" customHeight="1">
+    <row r="174" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
       <c r="D174" s="3"/>
       <c r="F174" s="3"/>
     </row>
-    <row r="175" ht="15.75" customHeight="1">
+    <row r="175" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
       <c r="F175" s="3"/>
     </row>
-    <row r="176" ht="15.75" customHeight="1">
+    <row r="176" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
       <c r="F176" s="3"/>
     </row>
-    <row r="177" ht="15.75" customHeight="1">
+    <row r="177" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
       <c r="D177" s="3"/>
       <c r="F177" s="3"/>
     </row>
-    <row r="178" ht="15.75" customHeight="1">
+    <row r="178" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
       <c r="D178" s="3"/>
       <c r="F178" s="3"/>
     </row>
-    <row r="179" ht="15.75" customHeight="1">
+    <row r="179" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
       <c r="D179" s="3"/>
       <c r="F179" s="3"/>
     </row>
-    <row r="180" ht="15.75" customHeight="1">
+    <row r="180" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
       <c r="D180" s="3"/>
       <c r="F180" s="3"/>
     </row>
-    <row r="181" ht="15.75" customHeight="1">
+    <row r="181" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
       <c r="D181" s="3"/>
       <c r="F181" s="3"/>
     </row>
-    <row r="182" ht="15.75" customHeight="1">
+    <row r="182" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
       <c r="D182" s="3"/>
       <c r="F182" s="3"/>
     </row>
-    <row r="183" ht="15.75" customHeight="1">
+    <row r="183" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
       <c r="D183" s="3"/>
       <c r="F183" s="3"/>
     </row>
-    <row r="184" ht="15.75" customHeight="1">
+    <row r="184" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
       <c r="D184" s="3"/>
       <c r="F184" s="3"/>
     </row>
-    <row r="185" ht="15.75" customHeight="1">
+    <row r="185" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
       <c r="D185" s="3"/>
       <c r="F185" s="3"/>
     </row>
-    <row r="186" ht="15.75" customHeight="1">
+    <row r="186" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
       <c r="D186" s="3"/>
       <c r="F186" s="3"/>
     </row>
-    <row r="187" ht="15.75" customHeight="1">
+    <row r="187" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
       <c r="D187" s="3"/>
       <c r="F187" s="3"/>
     </row>
-    <row r="188" ht="15.75" customHeight="1">
+    <row r="188" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
       <c r="D188" s="3"/>
       <c r="F188" s="3"/>
     </row>
-    <row r="189" ht="15.75" customHeight="1">
+    <row r="189" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
       <c r="D189" s="3"/>
       <c r="F189" s="3"/>
     </row>
-    <row r="190" ht="15.75" customHeight="1">
+    <row r="190" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
       <c r="D190" s="3"/>
       <c r="F190" s="3"/>
     </row>
-    <row r="191" ht="15.75" customHeight="1">
+    <row r="191" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
       <c r="D191" s="3"/>
       <c r="F191" s="3"/>
     </row>
-    <row r="192" ht="15.75" customHeight="1">
+    <row r="192" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
       <c r="D192" s="3"/>
       <c r="F192" s="3"/>
     </row>
-    <row r="193" ht="15.75" customHeight="1">
+    <row r="193" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
       <c r="D193" s="3"/>
       <c r="F193" s="3"/>
     </row>
-    <row r="194" ht="15.75" customHeight="1">
+    <row r="194" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
       <c r="D194" s="3"/>
       <c r="F194" s="3"/>
     </row>
-    <row r="195" ht="15.75" customHeight="1">
+    <row r="195" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
       <c r="D195" s="3"/>
       <c r="F195" s="3"/>
     </row>
-    <row r="196" ht="15.75" customHeight="1">
+    <row r="196" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
       <c r="D196" s="3"/>
       <c r="F196" s="3"/>
     </row>
-    <row r="197" ht="15.75" customHeight="1">
+    <row r="197" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
       <c r="D197" s="3"/>
       <c r="F197" s="3"/>
     </row>
-    <row r="198" ht="15.75" customHeight="1">
+    <row r="198" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
       <c r="D198" s="3"/>
       <c r="F198" s="3"/>
     </row>
-    <row r="199" ht="15.75" customHeight="1">
+    <row r="199" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
       <c r="F199" s="3"/>
     </row>
-    <row r="200" ht="15.75" customHeight="1">
+    <row r="200" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
       <c r="D200" s="3"/>
       <c r="F200" s="3"/>
     </row>
-    <row r="201" ht="15.75" customHeight="1">
+    <row r="201" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B201" s="3"/>
       <c r="C201" s="3"/>
       <c r="D201" s="3"/>
       <c r="F201" s="3"/>
     </row>
-    <row r="202" ht="15.75" customHeight="1">
+    <row r="202" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B202" s="3"/>
       <c r="C202" s="3"/>
       <c r="D202" s="3"/>
       <c r="F202" s="3"/>
     </row>
-    <row r="203" ht="15.75" customHeight="1">
+    <row r="203" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B203" s="3"/>
       <c r="C203" s="3"/>
       <c r="D203" s="3"/>
       <c r="F203" s="3"/>
     </row>
-    <row r="204" ht="15.75" customHeight="1">
+    <row r="204" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B204" s="3"/>
       <c r="C204" s="3"/>
       <c r="D204" s="3"/>
       <c r="F204" s="3"/>
     </row>
-    <row r="205" ht="15.75" customHeight="1">
+    <row r="205" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B205" s="3"/>
       <c r="C205" s="3"/>
       <c r="D205" s="3"/>
       <c r="F205" s="3"/>
     </row>
-    <row r="206" ht="15.75" customHeight="1">
+    <row r="206" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B206" s="3"/>
       <c r="C206" s="3"/>
       <c r="D206" s="3"/>
       <c r="F206" s="3"/>
     </row>
-    <row r="207" ht="15.75" customHeight="1">
+    <row r="207" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B207" s="3"/>
       <c r="C207" s="3"/>
       <c r="D207" s="3"/>
       <c r="F207" s="3"/>
     </row>
-    <row r="208" ht="15.75" customHeight="1">
+    <row r="208" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B208" s="3"/>
       <c r="C208" s="3"/>
       <c r="D208" s="3"/>
       <c r="F208" s="3"/>
     </row>
-    <row r="209" ht="15.75" customHeight="1">
+    <row r="209" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B209" s="3"/>
       <c r="C209" s="3"/>
       <c r="D209" s="3"/>
       <c r="F209" s="3"/>
     </row>
-    <row r="210" ht="15.75" customHeight="1">
+    <row r="210" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B210" s="3"/>
       <c r="C210" s="3"/>
       <c r="D210" s="3"/>
       <c r="F210" s="3"/>
     </row>
-    <row r="211" ht="15.75" customHeight="1">
+    <row r="211" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B211" s="3"/>
       <c r="C211" s="3"/>
       <c r="D211" s="3"/>
       <c r="F211" s="3"/>
     </row>
-    <row r="212" ht="15.75" customHeight="1">
+    <row r="212" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B212" s="3"/>
       <c r="C212" s="3"/>
       <c r="D212" s="3"/>
       <c r="F212" s="3"/>
     </row>
-    <row r="213" ht="15.75" customHeight="1">
+    <row r="213" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B213" s="3"/>
       <c r="C213" s="3"/>
       <c r="D213" s="3"/>
       <c r="F213" s="3"/>
     </row>
-    <row r="214" ht="15.75" customHeight="1">
+    <row r="214" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B214" s="3"/>
       <c r="C214" s="3"/>
       <c r="D214" s="3"/>
       <c r="F214" s="3"/>
     </row>
-    <row r="215" ht="15.75" customHeight="1">
+    <row r="215" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B215" s="3"/>
       <c r="C215" s="3"/>
       <c r="D215" s="3"/>
       <c r="F215" s="3"/>
     </row>
-    <row r="216" ht="15.75" customHeight="1">
+    <row r="216" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B216" s="3"/>
       <c r="C216" s="3"/>
       <c r="D216" s="3"/>
       <c r="F216" s="3"/>
     </row>
-    <row r="217" ht="15.75" customHeight="1">
+    <row r="217" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B217" s="3"/>
       <c r="C217" s="3"/>
       <c r="D217" s="3"/>
       <c r="F217" s="3"/>
     </row>
-    <row r="218" ht="15.75" customHeight="1">
+    <row r="218" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B218" s="3"/>
       <c r="C218" s="3"/>
       <c r="D218" s="3"/>
       <c r="F218" s="3"/>
     </row>
-    <row r="219" ht="15.75" customHeight="1">
+    <row r="219" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B219" s="3"/>
       <c r="C219" s="3"/>
       <c r="D219" s="3"/>
       <c r="F219" s="3"/>
     </row>
-    <row r="220" ht="15.75" customHeight="1">
+    <row r="220" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B220" s="3"/>
       <c r="C220" s="3"/>
       <c r="D220" s="3"/>
       <c r="F220" s="3"/>
     </row>
-    <row r="221" ht="15.75" customHeight="1">
+    <row r="221" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B221" s="3"/>
       <c r="C221" s="3"/>
       <c r="D221" s="3"/>
       <c r="F221" s="3"/>
     </row>
-    <row r="222" ht="15.75" customHeight="1">
+    <row r="222" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B222" s="3"/>
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
       <c r="F222" s="3"/>
     </row>
-    <row r="223" ht="15.75" customHeight="1">
+    <row r="223" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B223" s="3"/>
       <c r="C223" s="3"/>
       <c r="D223" s="3"/>
       <c r="F223" s="3"/>
     </row>
-    <row r="224" ht="15.75" customHeight="1">
+    <row r="224" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B224" s="3"/>
       <c r="C224" s="3"/>
       <c r="D224" s="3"/>
       <c r="F224" s="3"/>
     </row>
-    <row r="225" ht="15.75" customHeight="1">
+    <row r="225" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B225" s="3"/>
       <c r="C225" s="3"/>
       <c r="D225" s="3"/>
       <c r="F225" s="3"/>
     </row>
-    <row r="226" ht="15.75" customHeight="1">
+    <row r="226" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B226" s="3"/>
       <c r="C226" s="3"/>
       <c r="D226" s="3"/>
       <c r="F226" s="3"/>
     </row>
-    <row r="227" ht="15.75" customHeight="1">
+    <row r="227" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B227" s="3"/>
       <c r="C227" s="3"/>
       <c r="D227" s="3"/>
       <c r="F227" s="3"/>
     </row>
-    <row r="228" ht="15.75" customHeight="1">
+    <row r="228" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B228" s="3"/>
       <c r="C228" s="3"/>
       <c r="D228" s="3"/>
       <c r="F228" s="3"/>
     </row>
-    <row r="229" ht="15.75" customHeight="1">
+    <row r="229" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B229" s="3"/>
       <c r="C229" s="3"/>
       <c r="D229" s="3"/>
       <c r="F229" s="3"/>
     </row>
-    <row r="230" ht="15.75" customHeight="1">
+    <row r="230" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B230" s="3"/>
       <c r="C230" s="3"/>
       <c r="D230" s="3"/>
       <c r="F230" s="3"/>
     </row>
-    <row r="231" ht="15.75" customHeight="1">
+    <row r="231" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B231" s="3"/>
       <c r="C231" s="3"/>
       <c r="D231" s="3"/>
       <c r="F231" s="3"/>
     </row>
-    <row r="232" ht="15.75" customHeight="1">
+    <row r="232" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B232" s="3"/>
       <c r="C232" s="3"/>
       <c r="D232" s="3"/>
       <c r="F232" s="3"/>
     </row>
-    <row r="233" ht="15.75" customHeight="1">
+    <row r="233" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B233" s="3"/>
       <c r="C233" s="3"/>
       <c r="D233" s="3"/>
       <c r="F233" s="3"/>
     </row>
-    <row r="234" ht="15.75" customHeight="1">
+    <row r="234" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B234" s="3"/>
       <c r="C234" s="3"/>
       <c r="D234" s="3"/>
       <c r="F234" s="3"/>
     </row>
-    <row r="235" ht="15.75" customHeight="1">
+    <row r="235" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B235" s="3"/>
       <c r="C235" s="3"/>
       <c r="D235" s="3"/>
       <c r="F235" s="3"/>
     </row>
-    <row r="236" ht="15.75" customHeight="1">
+    <row r="236" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B236" s="3"/>
       <c r="C236" s="3"/>
       <c r="D236" s="3"/>
       <c r="F236" s="3"/>
     </row>
-    <row r="237" ht="15.75" customHeight="1">
+    <row r="237" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B237" s="3"/>
       <c r="C237" s="3"/>
       <c r="D237" s="3"/>
       <c r="F237" s="3"/>
     </row>
-    <row r="238" ht="15.75" customHeight="1">
+    <row r="238" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B238" s="3"/>
       <c r="C238" s="3"/>
       <c r="D238" s="3"/>
       <c r="F238" s="3"/>
     </row>
-    <row r="239" ht="15.75" customHeight="1">
+    <row r="239" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B239" s="3"/>
       <c r="C239" s="3"/>
       <c r="D239" s="3"/>
       <c r="F239" s="3"/>
     </row>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="240" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B10"/>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <printOptions gridLines="1" horizontalCentered="1"/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup fitToHeight="0" paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
-  <drawing r:id="rId2"/>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
 </worksheet>
 </file>
</xml_diff>